<commit_message>
update: v5 — 500K=pitch-baseline, 1M=2x scale, AT exclusivity
</commit_message>
<xml_diff>
--- a/GroundUP_BE_Szenarien_2030.xlsx
+++ b/GroundUP_BE_Szenarien_2030.xlsx
@@ -54,7 +54,7 @@
       <name val="Calibri"/>
       <b val="1"/>
       <color rgb="FFFFFFFF"/>
-      <sz val="9"/>
+      <sz val="10"/>
     </font>
     <font>
       <name val="Calibri"/>
@@ -65,19 +65,18 @@
     </font>
     <font>
       <name val="Calibri"/>
-      <b val="1"/>
       <color rgb="FF1A1A1A"/>
       <sz val="10"/>
     </font>
     <font>
       <name val="Calibri"/>
-      <color rgb="FF1A1A1A"/>
+      <color rgb="FF626567"/>
       <sz val="10"/>
     </font>
     <font>
       <name val="Calibri"/>
       <b val="1"/>
-      <color rgb="FF626567"/>
+      <color rgb="FF1A1A1A"/>
       <sz val="10"/>
     </font>
     <font>
@@ -88,6 +87,7 @@
     </font>
     <font>
       <name val="Calibri"/>
+      <b val="1"/>
       <color rgb="FF626567"/>
       <sz val="10"/>
     </font>
@@ -123,14 +123,14 @@
     <font>
       <name val="Calibri"/>
       <b val="1"/>
-      <color rgb="FF1A1A1A"/>
-      <sz val="11"/>
+      <color rgb="FFFFFFFF"/>
+      <sz val="9"/>
     </font>
     <font>
       <name val="Calibri"/>
       <b val="1"/>
-      <color rgb="FFFFFFFF"/>
-      <sz val="10"/>
+      <color rgb="FF1A1A1A"/>
+      <sz val="11"/>
     </font>
     <font>
       <name val="Calibri"/>
@@ -261,7 +261,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="68">
+  <cellXfs count="71">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -293,43 +293,43 @@
     <xf numFmtId="0" fontId="6" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="7" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="6" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="8" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="8" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="10" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="11" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="11" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="12" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="13" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -341,13 +341,16 @@
     <xf numFmtId="0" fontId="15" fillId="10" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="16" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="4" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="18" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -371,7 +374,7 @@
     <xf numFmtId="0" fontId="20" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="8" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="19" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -389,7 +392,10 @@
     <xf numFmtId="0" fontId="15" fillId="12" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="16" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -398,7 +404,7 @@
     <xf numFmtId="0" fontId="20" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="8" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="19" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -440,7 +446,10 @@
     <xf numFmtId="0" fontId="13" fillId="9" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="16" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -449,7 +458,7 @@
     <xf numFmtId="0" fontId="20" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="8" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="19" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -829,7 +838,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D31"/>
+  <dimension ref="A1:D37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="36" customWidth="1" min="1" max="1"/>
@@ -848,11 +857,11 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Kreditpreis an BE: 86 €/t  ·  BE Break-even: 100 €/t  ·  Zielpreis: 150 €/t  ·  April 2026</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="40" customHeight="1">
+          <t>Kreditpreis an BE: 86 €/t  ·  BE Break-even: 100 €/t  ·  BE Ziel: 150 €/t  ·  April 2026  ·  Pitch-Basis = 500K-Szenario</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="48" customHeight="1">
       <c r="A4" s="3" t="inlineStr">
         <is>
           <t>Kennzahl</t>
@@ -861,514 +870,634 @@
       <c r="B4" s="4" t="inlineStr">
         <is>
           <t>100K
-Pilotprogramm — Erster Zertifikatsverkauf 2029</t>
+Pilotpaket</t>
         </is>
       </c>
       <c r="C4" s="5" t="inlineStr">
         <is>
           <t>500K
-Vollständiger Burgenland-Rollout · +50% Enrollment-Wachstum 2029</t>
+Regionaler Ausbau
+(= Pitch-Basis)</t>
         </is>
       </c>
       <c r="D4" s="6" t="inlineStr">
         <is>
-          <t>1M  ⭐ AT-Exklusivität
-AT-Markt-Exklusivität · +100% Enrollment-Wachstum 2029</t>
+          <t>1M
+AT-Exklusivität
+⭐ 2× Scale</t>
         </is>
       </c>
     </row>
     <row r="5" ht="16" customHeight="1">
       <c r="A5" s="7" t="inlineStr">
         <is>
-          <t>── TRANCHE 1</t>
+          <t>── PHASE 1 (Q2 2026 – Q1 2027) · identisch für 500K und 1M</t>
         </is>
       </c>
     </row>
     <row r="6" ht="22" customHeight="1">
       <c r="A6" s="8" t="inlineStr">
         <is>
-          <t>Erster Zertifikatsverkauf (T1)</t>
+          <t>Q3 2026: Leitbetriebe / Testfläche</t>
         </is>
       </c>
       <c r="B6" s="9" t="inlineStr">
         <is>
-          <t>2029</t>
+          <t>10 Betriebe / ~2.000 ha</t>
         </is>
       </c>
       <c r="C6" s="9" t="inlineStr">
         <is>
-          <t>Q2/Q3 2027</t>
+          <t>10 Betriebe / 1.000–3.000 ha</t>
         </is>
       </c>
       <c r="D6" s="9" t="inlineStr">
         <is>
-          <t>Q2/Q3 2027</t>
+          <t>10 Betriebe / 1.000–3.000 ha</t>
         </is>
       </c>
     </row>
     <row r="7" ht="22" customHeight="1">
       <c r="A7" s="10" t="inlineStr">
         <is>
+          <t>Q4 2026: Onboarding-Kampagne</t>
+        </is>
+      </c>
+      <c r="B7" s="11" t="inlineStr">
+        <is>
+          <t>Phase läuft weiter</t>
+        </is>
+      </c>
+      <c r="C7" s="12" t="inlineStr">
+        <is>
+          <t>~100 neue Betriebe</t>
+        </is>
+      </c>
+      <c r="D7" s="12" t="inlineStr">
+        <is>
+          <t>~100 neue Betriebe</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="22" customHeight="1">
+      <c r="A8" s="8" t="inlineStr">
+        <is>
+          <t>Q1 2027: Aktiv / ha / PDD</t>
+        </is>
+      </c>
+      <c r="B8" s="13" t="inlineStr">
+        <is>
+          <t>Noch in Vorbereitung</t>
+        </is>
+      </c>
+      <c r="C8" s="9" t="inlineStr">
+        <is>
+          <t>100 Betriebe · 10.000 ha · PDD</t>
+        </is>
+      </c>
+      <c r="D8" s="9" t="inlineStr">
+        <is>
+          <t>100 Betriebe · 10.000 ha · PDD</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="16" customHeight="1">
+      <c r="A9" s="7" t="inlineStr">
+        <is>
+          <t>── TRANCHE 1</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="22" customHeight="1">
+      <c r="A10" s="14" t="inlineStr">
+        <is>
+          <t>Erster Zertifikatsverkauf</t>
+        </is>
+      </c>
+      <c r="B10" s="15" t="inlineStr">
+        <is>
+          <t>2029</t>
+        </is>
+      </c>
+      <c r="C10" s="16" t="inlineStr">
+        <is>
+          <t>✅ Q2/Q3 2027</t>
+        </is>
+      </c>
+      <c r="D10" s="16" t="inlineStr">
+        <is>
+          <t>✅ Q2/Q3 2027</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="22" customHeight="1">
+      <c r="A11" s="17" t="inlineStr">
+        <is>
           <t>Tonnen Tranche 1</t>
         </is>
       </c>
-      <c r="B7" s="11" t="inlineStr">
+      <c r="B11" s="18" t="inlineStr">
         <is>
           <t>5.000 t</t>
         </is>
       </c>
-      <c r="C7" s="11" t="inlineStr">
+      <c r="C11" s="18" t="inlineStr">
         <is>
           <t>5.000 t</t>
         </is>
       </c>
-      <c r="D7" s="11" t="inlineStr">
+      <c r="D11" s="18" t="inlineStr">
         <is>
           <t>5.000 t</t>
         </is>
       </c>
     </row>
-    <row r="8" ht="22" customHeight="1">
-      <c r="A8" s="12" t="inlineStr">
-        <is>
-          <t>Einkauf BE @ 86€/t</t>
-        </is>
-      </c>
-      <c r="B8" s="13" t="inlineStr">
+    <row r="12" ht="22" customHeight="1">
+      <c r="A12" s="10" t="inlineStr">
+        <is>
+          <t>Erlös BE @ 86€/t  (T1 Einkauf)</t>
+        </is>
+      </c>
+      <c r="B12" s="12" t="inlineStr">
         <is>
           <t>430,000 €</t>
         </is>
       </c>
-      <c r="C8" s="13" t="inlineStr">
+      <c r="C12" s="12" t="inlineStr">
         <is>
           <t>430,000 €</t>
         </is>
       </c>
-      <c r="D8" s="13" t="inlineStr">
+      <c r="D12" s="12" t="inlineStr">
         <is>
           <t>430,000 €</t>
         </is>
       </c>
     </row>
-    <row r="9" ht="22" customHeight="1">
-      <c r="A9" s="14" t="inlineStr">
-        <is>
-          <t>Marge BE @ 100€/t</t>
-        </is>
-      </c>
-      <c r="B9" s="15" t="inlineStr">
+    <row r="13" ht="22" customHeight="1">
+      <c r="A13" s="8" t="inlineStr">
+        <is>
+          <t>Marge BE @ 100€/t  (T1)</t>
+        </is>
+      </c>
+      <c r="B13" s="9" t="inlineStr">
         <is>
           <t>70,000 €</t>
         </is>
       </c>
-      <c r="C9" s="15" t="inlineStr">
+      <c r="C13" s="9" t="inlineStr">
         <is>
           <t>70,000 €</t>
         </is>
       </c>
-      <c r="D9" s="15" t="inlineStr">
+      <c r="D13" s="9" t="inlineStr">
         <is>
           <t>70,000 €</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="22" customHeight="1">
-      <c r="A10" s="12" t="inlineStr">
-        <is>
-          <t>Marge BE @ 150€/t</t>
-        </is>
-      </c>
-      <c r="B10" s="13" t="inlineStr">
-        <is>
-          <t>320,000 €</t>
-        </is>
-      </c>
-      <c r="C10" s="13" t="inlineStr">
-        <is>
-          <t>320,000 €</t>
-        </is>
-      </c>
-      <c r="D10" s="13" t="inlineStr">
-        <is>
-          <t>320,000 €</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" ht="16" customHeight="1">
-      <c r="A11" s="7" t="inlineStr">
-        <is>
-          <t>── ENROLLMENT-WACHSTUM &amp; PORTFOLIO-AUFBAU</t>
-        </is>
-      </c>
-    </row>
-    <row r="12" ht="22" customHeight="1">
-      <c r="A12" s="14" t="inlineStr">
-        <is>
-          <t>Betriebe 2028 (kumuliert)</t>
-        </is>
-      </c>
-      <c r="B12" s="15" t="inlineStr">
-        <is>
-          <t>50 Betriebe</t>
-        </is>
-      </c>
-      <c r="C12" s="15" t="inlineStr">
-        <is>
-          <t>300 Betriebe</t>
-        </is>
-      </c>
-      <c r="D12" s="15" t="inlineStr">
-        <is>
-          <t>500 Betriebe</t>
-        </is>
-      </c>
-    </row>
-    <row r="13" ht="22" customHeight="1">
-      <c r="A13" s="12" t="inlineStr">
-        <is>
-          <t>Hektar 2028 (kumuliert)</t>
-        </is>
-      </c>
-      <c r="B13" s="13" t="inlineStr">
-        <is>
-          <t>4,000 ha</t>
-        </is>
-      </c>
-      <c r="C13" s="13" t="inlineStr">
-        <is>
-          <t>30,000 ha</t>
-        </is>
-      </c>
-      <c r="D13" s="13" t="inlineStr">
-        <is>
-          <t>60,000 ha</t>
         </is>
       </c>
     </row>
     <row r="14" ht="22" customHeight="1">
       <c r="A14" s="10" t="inlineStr">
         <is>
-          <t>Enrollment-Wachstum 2029</t>
-        </is>
-      </c>
-      <c r="B14" s="16" t="inlineStr">
-        <is>
-          <t>Tranche 2 in Vorbereitung</t>
-        </is>
-      </c>
-      <c r="C14" s="17" t="inlineStr">
-        <is>
-          <t>+50% ggü. 2027</t>
-        </is>
-      </c>
-      <c r="D14" s="17" t="inlineStr">
-        <is>
-          <t>+100% ggü. 2027</t>
+          <t>Marge BE @ 150€/t  (T1)</t>
+        </is>
+      </c>
+      <c r="B14" s="12" t="inlineStr">
+        <is>
+          <t>320,000 €</t>
+        </is>
+      </c>
+      <c r="C14" s="12" t="inlineStr">
+        <is>
+          <t>320,000 €</t>
+        </is>
+      </c>
+      <c r="D14" s="12" t="inlineStr">
+        <is>
+          <t>320,000 €</t>
         </is>
       </c>
     </row>
     <row r="15" ht="16" customHeight="1">
       <c r="A15" s="7" t="inlineStr">
         <is>
-          <t>── TRANCHE 2</t>
+          <t>── PORTFOLIO-AUFBAU &amp; SKALIERUNG 2028</t>
         </is>
       </c>
     </row>
     <row r="16" ht="22" customHeight="1">
-      <c r="A16" s="8" t="inlineStr">
-        <is>
-          <t>Tranche 2</t>
+      <c r="A16" s="17" t="inlineStr">
+        <is>
+          <t>Betriebe 2028 (kumuliert)</t>
         </is>
       </c>
       <c r="B16" s="18" t="inlineStr">
         <is>
-          <t>—  (nach 2030)</t>
-        </is>
-      </c>
-      <c r="C16" s="19" t="inlineStr">
-        <is>
-          <t>25.000 t  (2029)</t>
+          <t>~50 Betriebe</t>
+        </is>
+      </c>
+      <c r="C16" s="18" t="inlineStr">
+        <is>
+          <t>500 Betriebe</t>
         </is>
       </c>
       <c r="D16" s="19" t="inlineStr">
         <is>
-          <t>50.000 t  (2029)</t>
+          <t>1.000 Betriebe</t>
         </is>
       </c>
     </row>
     <row r="17" ht="22" customHeight="1">
       <c r="A17" s="14" t="inlineStr">
         <is>
-          <t>Einkauf BE @ 86€/t  (T2)</t>
-        </is>
-      </c>
-      <c r="B17" s="20" t="inlineStr">
-        <is>
-          <t>—</t>
+          <t>Hektar 2028 (kumuliert)</t>
+        </is>
+      </c>
+      <c r="B17" s="15" t="inlineStr">
+        <is>
+          <t>~4.000 ha</t>
         </is>
       </c>
       <c r="C17" s="15" t="inlineStr">
         <is>
+          <t>50.000+ ha</t>
+        </is>
+      </c>
+      <c r="D17" s="15" t="inlineStr">
+        <is>
+          <t>100.000+ ha</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="16" customHeight="1">
+      <c r="A18" s="7" t="inlineStr">
+        <is>
+          <t>── TRANCHE 2 (2029)</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="22" customHeight="1">
+      <c r="A19" s="17" t="inlineStr">
+        <is>
+          <t>Tonnen Tranche 2</t>
+        </is>
+      </c>
+      <c r="B19" s="20" t="inlineStr">
+        <is>
+          <t>— (nach 2030)</t>
+        </is>
+      </c>
+      <c r="C19" s="18" t="inlineStr">
+        <is>
+          <t>25.000 t</t>
+        </is>
+      </c>
+      <c r="D19" s="19" t="inlineStr">
+        <is>
+          <t>50.000 t</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="22" customHeight="1">
+      <c r="A20" s="10" t="inlineStr">
+        <is>
+          <t>Betriebe bei T2</t>
+        </is>
+      </c>
+      <c r="B20" s="11" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="C20" s="12" t="inlineStr">
+        <is>
+          <t>750 Betriebe</t>
+        </is>
+      </c>
+      <c r="D20" s="21" t="inlineStr">
+        <is>
+          <t>1.500 Betriebe</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="22" customHeight="1">
+      <c r="A21" s="8" t="inlineStr">
+        <is>
+          <t>Erlös BE @ 86€/t  (T2 Einkauf)</t>
+        </is>
+      </c>
+      <c r="B21" s="13" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="C21" s="9" t="inlineStr">
+        <is>
           <t>2,150,000 €</t>
         </is>
       </c>
-      <c r="D17" s="15" t="inlineStr">
+      <c r="D21" s="9" t="inlineStr">
         <is>
           <t>4,300,000 €</t>
         </is>
       </c>
     </row>
-    <row r="18" ht="22" customHeight="1">
-      <c r="A18" s="12" t="inlineStr">
+    <row r="22" ht="22" customHeight="1">
+      <c r="A22" s="10" t="inlineStr">
+        <is>
+          <t>Umsatz BE @ 100€/t  (T2)</t>
+        </is>
+      </c>
+      <c r="B22" s="11" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="C22" s="21" t="inlineStr">
+        <is>
+          <t>2,5 Mio €</t>
+        </is>
+      </c>
+      <c r="D22" s="21" t="inlineStr">
+        <is>
+          <t>5,0 Mio €</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="22" customHeight="1">
+      <c r="A23" s="8" t="inlineStr">
+        <is>
+          <t>Umsatz BE @ 150€/t  (T2)</t>
+        </is>
+      </c>
+      <c r="B23" s="13" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="C23" s="22" t="inlineStr">
+        <is>
+          <t>3,75 Mio €</t>
+        </is>
+      </c>
+      <c r="D23" s="22" t="inlineStr">
+        <is>
+          <t>7,5 Mio €</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="22" customHeight="1">
+      <c r="A24" s="10" t="inlineStr">
         <is>
           <t>Marge BE @ 100€/t  (T2)</t>
         </is>
       </c>
-      <c r="B18" s="21" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="C18" s="13" t="inlineStr">
+      <c r="B24" s="11" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="C24" s="12" t="inlineStr">
         <is>
           <t>350,000 €</t>
         </is>
       </c>
-      <c r="D18" s="13" t="inlineStr">
+      <c r="D24" s="12" t="inlineStr">
         <is>
           <t>700,000 €</t>
         </is>
       </c>
     </row>
-    <row r="19" ht="22" customHeight="1">
-      <c r="A19" s="14" t="inlineStr">
+    <row r="25" ht="22" customHeight="1">
+      <c r="A25" s="17" t="inlineStr">
         <is>
           <t>Marge BE @ 150€/t  (T2)</t>
         </is>
       </c>
-      <c r="B19" s="20" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="C19" s="15" t="inlineStr">
+      <c r="B25" s="20" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="C25" s="18" t="inlineStr">
         <is>
           <t>1,600,000 €</t>
         </is>
       </c>
-      <c r="D19" s="15" t="inlineStr">
+      <c r="D25" s="18" t="inlineStr">
         <is>
           <t>3,200,000 €</t>
         </is>
       </c>
     </row>
-    <row r="20" ht="16" customHeight="1">
-      <c r="A20" s="7" t="inlineStr">
+    <row r="26" ht="16" customHeight="1">
+      <c r="A26" s="7" t="inlineStr">
         <is>
           <t>── AB 2030: JÄHRLICHES ERNTEN</t>
-        </is>
-      </c>
-    </row>
-    <row r="21" ht="22" customHeight="1">
-      <c r="A21" s="12" t="inlineStr">
-        <is>
-          <t>Jährl. Tonnen ab 2030+</t>
-        </is>
-      </c>
-      <c r="B21" s="21" t="inlineStr">
-        <is>
-          <t>gering</t>
-        </is>
-      </c>
-      <c r="C21" s="22" t="inlineStr">
-        <is>
-          <t>~12.000 t/yr</t>
-        </is>
-      </c>
-      <c r="D21" s="22" t="inlineStr">
-        <is>
-          <t>~32.000 t/yr</t>
-        </is>
-      </c>
-    </row>
-    <row r="22" ht="22" customHeight="1">
-      <c r="A22" s="14" t="inlineStr">
-        <is>
-          <t>Jährl. Marge BE @ 150€/t</t>
-        </is>
-      </c>
-      <c r="B22" s="20" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="C22" s="15" t="inlineStr">
-        <is>
-          <t>~768,000 €/yr</t>
-        </is>
-      </c>
-      <c r="D22" s="15" t="inlineStr">
-        <is>
-          <t>~2,048,000 €/yr</t>
-        </is>
-      </c>
-    </row>
-    <row r="23" ht="16" customHeight="1">
-      <c r="A23" s="7" t="inlineStr">
-        <is>
-          <t>── KUMULIERT T1 + T2 (BIS 2029)</t>
-        </is>
-      </c>
-    </row>
-    <row r="24" ht="22" customHeight="1">
-      <c r="A24" s="8" t="inlineStr">
-        <is>
-          <t>Gesamtinvestment BE</t>
-        </is>
-      </c>
-      <c r="B24" s="9" t="inlineStr">
-        <is>
-          <t>100,000 €</t>
-        </is>
-      </c>
-      <c r="C24" s="9" t="inlineStr">
-        <is>
-          <t>500,000 €</t>
-        </is>
-      </c>
-      <c r="D24" s="9" t="inlineStr">
-        <is>
-          <t>1,000,000 €</t>
-        </is>
-      </c>
-    </row>
-    <row r="25" ht="22" customHeight="1">
-      <c r="A25" s="10" t="inlineStr">
-        <is>
-          <t>Kum. Tonnen T1+T2</t>
-        </is>
-      </c>
-      <c r="B25" s="11" t="inlineStr">
-        <is>
-          <t>5.000 t  (2029)</t>
-        </is>
-      </c>
-      <c r="C25" s="17" t="inlineStr">
-        <is>
-          <t>30.000 t</t>
-        </is>
-      </c>
-      <c r="D25" s="17" t="inlineStr">
-        <is>
-          <t>55.000 t</t>
-        </is>
-      </c>
-    </row>
-    <row r="26" ht="22" customHeight="1">
-      <c r="A26" s="12" t="inlineStr">
-        <is>
-          <t>Kum. Marge @ 100€/t</t>
-        </is>
-      </c>
-      <c r="B26" s="13" t="inlineStr">
-        <is>
-          <t>70,000 €</t>
-        </is>
-      </c>
-      <c r="C26" s="13" t="inlineStr">
-        <is>
-          <t>420,000 €</t>
-        </is>
-      </c>
-      <c r="D26" s="13" t="inlineStr">
-        <is>
-          <t>770,000 €</t>
         </is>
       </c>
     </row>
     <row r="27" ht="22" customHeight="1">
       <c r="A27" s="10" t="inlineStr">
         <is>
+          <t>Jährl. Tonnen ab 2030+</t>
+        </is>
+      </c>
+      <c r="B27" s="11" t="inlineStr">
+        <is>
+          <t>gering</t>
+        </is>
+      </c>
+      <c r="C27" s="12" t="inlineStr">
+        <is>
+          <t>~12.000 t/yr</t>
+        </is>
+      </c>
+      <c r="D27" s="21" t="inlineStr">
+        <is>
+          <t>~32.000 t/yr</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="22" customHeight="1">
+      <c r="A28" s="8" t="inlineStr">
+        <is>
+          <t>Jährl. Marge BE @ 150€/t</t>
+        </is>
+      </c>
+      <c r="B28" s="13" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="C28" s="9" t="inlineStr">
+        <is>
+          <t>~768,000 €/yr</t>
+        </is>
+      </c>
+      <c r="D28" s="9" t="inlineStr">
+        <is>
+          <t>~2,048,000 €/yr</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="16" customHeight="1">
+      <c r="A29" s="7" t="inlineStr">
+        <is>
+          <t>── KUMULIERT T1 + T2 (2027–2029)</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="22" customHeight="1">
+      <c r="A30" s="14" t="inlineStr">
+        <is>
+          <t>Gesamtinvestment BE</t>
+        </is>
+      </c>
+      <c r="B30" s="15" t="inlineStr">
+        <is>
+          <t>100.000 €</t>
+        </is>
+      </c>
+      <c r="C30" s="15" t="inlineStr">
+        <is>
+          <t>500.000 €</t>
+        </is>
+      </c>
+      <c r="D30" s="15" t="inlineStr">
+        <is>
+          <t>1.000.000 €</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="22" customHeight="1">
+      <c r="A31" s="17" t="inlineStr">
+        <is>
+          <t>Kum. Tonnen T1 + T2</t>
+        </is>
+      </c>
+      <c r="B31" s="18" t="inlineStr">
+        <is>
+          <t>5.000 t  (2029)</t>
+        </is>
+      </c>
+      <c r="C31" s="18" t="inlineStr">
+        <is>
+          <t>30.000 t</t>
+        </is>
+      </c>
+      <c r="D31" s="19" t="inlineStr">
+        <is>
+          <t>55.000 t</t>
+        </is>
+      </c>
+    </row>
+    <row r="32" ht="22" customHeight="1">
+      <c r="A32" s="10" t="inlineStr">
+        <is>
+          <t>Kum. Marge @ 100€/t</t>
+        </is>
+      </c>
+      <c r="B32" s="12" t="inlineStr">
+        <is>
+          <t>70,000 €</t>
+        </is>
+      </c>
+      <c r="C32" s="12" t="inlineStr">
+        <is>
+          <t>420,000 €</t>
+        </is>
+      </c>
+      <c r="D32" s="12" t="inlineStr">
+        <is>
+          <t>770,000 €</t>
+        </is>
+      </c>
+    </row>
+    <row r="33" ht="22" customHeight="1">
+      <c r="A33" s="17" t="inlineStr">
+        <is>
           <t>Kum. Marge @ 150€/t</t>
         </is>
       </c>
-      <c r="B27" s="11" t="inlineStr">
+      <c r="B33" s="18" t="inlineStr">
         <is>
           <t>320,000 €</t>
         </is>
       </c>
-      <c r="C27" s="11" t="inlineStr">
+      <c r="C33" s="18" t="inlineStr">
         <is>
           <t>1,920,000 €</t>
         </is>
       </c>
-      <c r="D27" s="11" t="inlineStr">
+      <c r="D33" s="18" t="inlineStr">
         <is>
           <t>3,520,000 €</t>
         </is>
       </c>
     </row>
-    <row r="28" ht="22" customHeight="1">
-      <c r="A28" s="12" t="inlineStr">
-        <is>
-          <t>CORSIA-fähige Credits ab</t>
-        </is>
-      </c>
-      <c r="B28" s="13" t="inlineStr">
+    <row r="34" ht="22" customHeight="1">
+      <c r="A34" s="10" t="inlineStr">
+        <is>
+          <t>CORSIA-fähig ab</t>
+        </is>
+      </c>
+      <c r="B34" s="12" t="inlineStr">
         <is>
           <t>2029</t>
         </is>
       </c>
-      <c r="C28" s="22" t="inlineStr">
+      <c r="C34" s="21" t="inlineStr">
         <is>
           <t>✅ Q2/Q3 2027</t>
         </is>
       </c>
-      <c r="D28" s="22" t="inlineStr">
+      <c r="D34" s="21" t="inlineStr">
         <is>
           <t>✅ Q2/Q3 2027</t>
         </is>
       </c>
     </row>
-    <row r="29" ht="22" customHeight="1">
-      <c r="A29" s="10" t="inlineStr">
-        <is>
-          <t>AT-Markt-Exklusivität für BE</t>
-        </is>
-      </c>
-      <c r="B29" s="16" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="C29" s="16" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="D29" s="23" t="inlineStr">
+    <row r="35" ht="22" customHeight="1">
+      <c r="A35" s="17" t="inlineStr">
+        <is>
+          <t>AT-Markt-Exklusivität</t>
+        </is>
+      </c>
+      <c r="B35" s="20" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="C35" s="20" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D35" s="23" t="inlineStr">
         <is>
           <t>⭐ Inklusive</t>
         </is>
       </c>
     </row>
-    <row r="31" ht="40" customHeight="1">
-      <c r="A31" s="24" t="inlineStr">
-        <is>
-          <t>⭐  Das 1M-Investment sichert Burgenland Energie die Exklusivität für den österreichischen Carbon-Farming-Markt. BE wird zum einzigen Anbieter von Verra-zertifizierten, regionalen Soil-Carbon-Credits in Österreich.</t>
+    <row r="37" ht="40" customHeight="1">
+      <c r="A37" s="24" t="inlineStr">
+        <is>
+          <t>⭐  Das 1M-Investment beinhaltet die Markt-Exklusivität für Burgenland Energie im gesamten österreichischen Carbon-Farming-Markt. BE wird zum einzigen Anbieter von Verra-zertifizierten, regionalen Soil-Carbon-Credits in Österreich.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="8">
+  <mergeCells count="9">
     <mergeCell ref="A1:D1"/>
     <mergeCell ref="A5:D5"/>
-    <mergeCell ref="A23:D23"/>
-    <mergeCell ref="A31:D31"/>
-    <mergeCell ref="A20:D20"/>
+    <mergeCell ref="A9:D9"/>
+    <mergeCell ref="A18:D18"/>
+    <mergeCell ref="A37:D37"/>
+    <mergeCell ref="A26:D26"/>
     <mergeCell ref="A15:D15"/>
+    <mergeCell ref="A29:D29"/>
     <mergeCell ref="A2:D2"/>
-    <mergeCell ref="A11:D11"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1385,7 +1514,7 @@
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
     <col width="32" customWidth="1" min="2" max="2"/>
-    <col width="38" customWidth="1" min="3" max="3"/>
+    <col width="40" customWidth="1" min="3" max="3"/>
     <col width="18" customWidth="1" min="4" max="4"/>
     <col width="18" customWidth="1" min="5" max="5"/>
   </cols>
@@ -1405,226 +1534,226 @@
       </c>
     </row>
     <row r="4" ht="20" customHeight="1">
-      <c r="A4" s="4" t="inlineStr">
+      <c r="A4" s="27" t="inlineStr">
         <is>
           <t>Gesamt-Investment</t>
         </is>
       </c>
-      <c r="B4" s="4" t="inlineStr">
+      <c r="B4" s="27" t="inlineStr">
         <is>
           <t>Tranche 1</t>
         </is>
       </c>
-      <c r="C4" s="4" t="inlineStr">
+      <c r="C4" s="27" t="inlineStr">
         <is>
           <t>Tranche 2</t>
         </is>
       </c>
-      <c r="D4" s="4" t="inlineStr">
+      <c r="D4" s="27" t="inlineStr">
         <is>
           <t>Betriebe 2028</t>
         </is>
       </c>
-      <c r="E4" s="4" t="inlineStr">
+      <c r="E4" s="27" t="inlineStr">
         <is>
           <t>Hektar 2028</t>
         </is>
       </c>
     </row>
-    <row r="5" ht="32" customHeight="1">
-      <c r="A5" s="27" t="inlineStr">
-        <is>
-          <t>100,000 €</t>
-        </is>
-      </c>
-      <c r="B5" s="27" t="inlineStr">
+    <row r="5" ht="34" customHeight="1">
+      <c r="A5" s="28" t="inlineStr">
+        <is>
+          <t>100.000 €</t>
+        </is>
+      </c>
+      <c r="B5" s="28" t="inlineStr">
         <is>
           <t>5.000 t
 (2029)</t>
         </is>
       </c>
-      <c r="C5" s="27" t="inlineStr">
+      <c r="C5" s="28" t="inlineStr">
         <is>
           <t>—
 (nach 2030)</t>
         </is>
       </c>
-      <c r="D5" s="27" t="inlineStr">
-        <is>
-          <t>50</t>
-        </is>
-      </c>
-      <c r="E5" s="27" t="inlineStr">
-        <is>
-          <t>4,000 ha</t>
+      <c r="D5" s="28" t="inlineStr">
+        <is>
+          <t>~50</t>
+        </is>
+      </c>
+      <c r="E5" s="28" t="inlineStr">
+        <is>
+          <t>~4.000 ha</t>
         </is>
       </c>
     </row>
     <row r="7" ht="26" customHeight="1">
-      <c r="A7" s="28" t="inlineStr">
-        <is>
-          <t>Meilensteinplan — aligned mit Pitch Burgenland Energie (2026–2030+)</t>
+      <c r="A7" s="29" t="inlineStr">
+        <is>
+          <t>Meilensteinplan — Ground UP × Burgenland Energie (2026–2030+)</t>
         </is>
       </c>
     </row>
     <row r="8" ht="22" customHeight="1">
-      <c r="A8" s="29" t="inlineStr">
+      <c r="A8" s="30" t="inlineStr">
         <is>
           <t>Phase</t>
         </is>
       </c>
-      <c r="B8" s="29" t="inlineStr">
+      <c r="B8" s="30" t="inlineStr">
         <is>
           <t>Milestone</t>
         </is>
       </c>
-      <c r="C8" s="29" t="inlineStr">
+      <c r="C8" s="30" t="inlineStr">
         <is>
           <t>Aktivitäten &amp; Deliverables</t>
         </is>
       </c>
-      <c r="D8" s="29" t="inlineStr">
+      <c r="D8" s="30" t="inlineStr">
         <is>
           <t>Tonnen</t>
         </is>
       </c>
-      <c r="E8" s="29" t="inlineStr">
+      <c r="E8" s="30" t="inlineStr">
         <is>
           <t>Erlös BE @ 86€</t>
         </is>
       </c>
     </row>
     <row r="9" ht="34" customHeight="1">
-      <c r="A9" s="30" t="inlineStr">
+      <c r="A9" s="31" t="inlineStr">
         <is>
           <t>2026
 Phase 1 Start</t>
         </is>
       </c>
-      <c r="B9" s="12" t="inlineStr">
-        <is>
-          <t>Pilotprogramm · Leitbetriebe</t>
-        </is>
-      </c>
-      <c r="C9" s="31" t="inlineStr">
-        <is>
-          <t>Partnerschaftsvertrag · 10 Leitbetriebe · MRV-Aufbau</t>
-        </is>
-      </c>
-      <c r="D9" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E9" s="32" t="inlineStr">
+      <c r="B9" s="8" t="inlineStr">
+        <is>
+          <t>Pilotprogramm · 10 Leitbetriebe</t>
+        </is>
+      </c>
+      <c r="C9" s="32" t="inlineStr">
+        <is>
+          <t>Partnerschaftsvertrag · MRV-Aufbau · erste Bodenproben &amp; Baseline</t>
+        </is>
+      </c>
+      <c r="D9" s="33" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E9" s="33" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
     </row>
     <row r="10" ht="34" customHeight="1">
-      <c r="A10" s="33" t="inlineStr">
+      <c r="A10" s="34" t="inlineStr">
         <is>
           <t>2027
 Vorbereitung</t>
         </is>
       </c>
-      <c r="B10" s="14" t="inlineStr">
-        <is>
-          <t>Verra-Dossier in Aufbau · Monitoring startet</t>
-        </is>
-      </c>
-      <c r="C10" s="34" t="inlineStr">
-        <is>
-          <t>Bodenproben · Historische Daten · Verra-Vorbereitung</t>
-        </is>
-      </c>
-      <c r="D10" s="35" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E10" s="35" t="inlineStr">
+      <c r="B10" s="10" t="inlineStr">
+        <is>
+          <t>Verra-Dossier in Aufbau · Monitoring-Phase startet</t>
+        </is>
+      </c>
+      <c r="C10" s="35" t="inlineStr">
+        <is>
+          <t>Historische Datenaufbereitung · Laboranalysen · Verra-Vorbereitung</t>
+        </is>
+      </c>
+      <c r="D10" s="36" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E10" s="36" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
     </row>
     <row r="11" ht="34" customHeight="1">
-      <c r="A11" s="30" t="inlineStr">
+      <c r="A11" s="31" t="inlineStr">
         <is>
           <t>2028
 Onboarding</t>
         </is>
       </c>
-      <c r="B11" s="12" t="inlineStr">
-        <is>
-          <t>Weitere Betriebe · Dossier-Fertigstellung</t>
-        </is>
-      </c>
-      <c r="C11" s="31" t="inlineStr">
-        <is>
-          <t>Vollständige Datenaufbereitung · PDD-Einreichung vorbereitet</t>
-        </is>
-      </c>
-      <c r="D11" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E11" s="32" t="inlineStr">
+      <c r="B11" s="8" t="inlineStr">
+        <is>
+          <t>~50 Betriebe · ~4.000 ha · PDD-Fertigstellung</t>
+        </is>
+      </c>
+      <c r="C11" s="32" t="inlineStr">
+        <is>
+          <t>Vollständige Dossier-Aufbereitung · PDD-Einreichung bei Verra</t>
+        </is>
+      </c>
+      <c r="D11" s="33" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E11" s="33" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
     </row>
     <row r="12" ht="34" customHeight="1">
-      <c r="A12" s="36" t="inlineStr">
+      <c r="A12" s="37" t="inlineStr">
         <is>
           <t>2029
 🎯 TRANCHE 1</t>
         </is>
       </c>
-      <c r="B12" s="37" t="inlineStr">
+      <c r="B12" s="38" t="inlineStr">
         <is>
           <t>Erster Zertifikatsverkauf · 5.000 t</t>
         </is>
       </c>
-      <c r="C12" s="38" t="inlineStr">
+      <c r="C12" s="39" t="inlineStr">
         <is>
           <t>Verra VCU-Issuance · CORSIA-fähige Credits für BE Trading</t>
         </is>
       </c>
-      <c r="D12" s="39" t="n">
+      <c r="D12" s="40" t="n">
         <v>5000</v>
       </c>
-      <c r="E12" s="40" t="n">
+      <c r="E12" s="41" t="n">
         <v>430000</v>
       </c>
     </row>
     <row r="13" ht="34" customHeight="1">
-      <c r="A13" s="30" t="inlineStr">
+      <c r="A13" s="31" t="inlineStr">
         <is>
           <t>2030
 Portfolio-Aufbau</t>
         </is>
       </c>
-      <c r="B13" s="12" t="inlineStr">
-        <is>
-          <t>Monitoring-Zyklus · Vorbereitung Tranche 2</t>
-        </is>
-      </c>
-      <c r="C13" s="31" t="inlineStr">
-        <is>
-          <t>Wachsendes Betriebsnetzwerk · Nächste Tranche in Planung</t>
-        </is>
-      </c>
-      <c r="D13" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E13" s="32" t="inlineStr">
+      <c r="B13" s="8" t="inlineStr">
+        <is>
+          <t>Monitoring-Zyklus · Nächste Tranche in Vorbereitung</t>
+        </is>
+      </c>
+      <c r="C13" s="32" t="inlineStr">
+        <is>
+          <t>Wachsendes Betriebsnetzwerk · Tranche 2 in Planung</t>
+        </is>
+      </c>
+      <c r="D13" s="33" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E13" s="33" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1646,381 +1775,409 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E21"/>
+  <dimension ref="A1:E22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
     <col width="32" customWidth="1" min="2" max="2"/>
-    <col width="38" customWidth="1" min="3" max="3"/>
+    <col width="40" customWidth="1" min="3" max="3"/>
     <col width="18" customWidth="1" min="4" max="4"/>
     <col width="18" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1" ht="34" customHeight="1">
-      <c r="A1" s="41" t="inlineStr">
+      <c r="A1" s="42" t="inlineStr">
         <is>
           <t>Ground UP × BE  ·  500K Regionaler Ausbau</t>
         </is>
       </c>
     </row>
     <row r="2" ht="18" customHeight="1">
-      <c r="A2" s="42" t="inlineStr">
-        <is>
-          <t>Vollständiger Burgenland-Rollout · +50% Enrollment-Wachstum 2029</t>
+      <c r="A2" s="43" t="inlineStr">
+        <is>
+          <t>Vollständiger Burgenland-Rollout  ·  Pitch-Zahlen BE</t>
         </is>
       </c>
     </row>
     <row r="4" ht="20" customHeight="1">
-      <c r="A4" s="5" t="inlineStr">
+      <c r="A4" s="44" t="inlineStr">
         <is>
           <t>Gesamt-Investment</t>
         </is>
       </c>
-      <c r="B4" s="5" t="inlineStr">
+      <c r="B4" s="44" t="inlineStr">
         <is>
           <t>Tranche 1</t>
         </is>
       </c>
-      <c r="C4" s="5" t="inlineStr">
+      <c r="C4" s="44" t="inlineStr">
         <is>
           <t>Tranche 2</t>
         </is>
       </c>
-      <c r="D4" s="5" t="inlineStr">
+      <c r="D4" s="44" t="inlineStr">
         <is>
           <t>Betriebe 2028</t>
         </is>
       </c>
-      <c r="E4" s="5" t="inlineStr">
+      <c r="E4" s="44" t="inlineStr">
         <is>
           <t>Hektar 2028</t>
         </is>
       </c>
     </row>
-    <row r="5" ht="32" customHeight="1">
-      <c r="A5" s="43" t="inlineStr">
-        <is>
-          <t>500,000 €</t>
-        </is>
-      </c>
-      <c r="B5" s="43" t="inlineStr">
+    <row r="5" ht="34" customHeight="1">
+      <c r="A5" s="45" t="inlineStr">
+        <is>
+          <t>500.000 €</t>
+        </is>
+      </c>
+      <c r="B5" s="45" t="inlineStr">
         <is>
           <t>5.000 t
 (Q2/Q3 2027)</t>
         </is>
       </c>
-      <c r="C5" s="43" t="inlineStr">
-        <is>
-          <t>25,000 t
+      <c r="C5" s="45" t="inlineStr">
+        <is>
+          <t>25.000 t
 (2029)</t>
         </is>
       </c>
-      <c r="D5" s="43" t="inlineStr">
-        <is>
-          <t>300</t>
-        </is>
-      </c>
-      <c r="E5" s="43" t="inlineStr">
-        <is>
-          <t>30,000 ha</t>
+      <c r="D5" s="45" t="inlineStr">
+        <is>
+          <t>500</t>
+        </is>
+      </c>
+      <c r="E5" s="45" t="inlineStr">
+        <is>
+          <t>50.000+ ha</t>
         </is>
       </c>
     </row>
     <row r="7" ht="26" customHeight="1">
-      <c r="A7" s="44" t="inlineStr">
-        <is>
-          <t>Meilensteinplan — aligned mit Pitch Burgenland Energie (2026–2030+)</t>
+      <c r="A7" s="46" t="inlineStr">
+        <is>
+          <t>Meilensteinplan — Ground UP × Burgenland Energie (2026–2030+)</t>
         </is>
       </c>
     </row>
     <row r="8" ht="22" customHeight="1">
-      <c r="A8" s="29" t="inlineStr">
+      <c r="A8" s="30" t="inlineStr">
         <is>
           <t>Phase</t>
         </is>
       </c>
-      <c r="B8" s="29" t="inlineStr">
+      <c r="B8" s="30" t="inlineStr">
         <is>
           <t>Milestone</t>
         </is>
       </c>
-      <c r="C8" s="29" t="inlineStr">
+      <c r="C8" s="30" t="inlineStr">
         <is>
           <t>Aktivitäten &amp; Deliverables</t>
         </is>
       </c>
-      <c r="D8" s="29" t="inlineStr">
+      <c r="D8" s="30" t="inlineStr">
         <is>
           <t>Tonnen</t>
         </is>
       </c>
-      <c r="E8" s="29" t="inlineStr">
+      <c r="E8" s="30" t="inlineStr">
         <is>
           <t>Erlös BE @ 86€</t>
         </is>
       </c>
     </row>
     <row r="9" ht="34" customHeight="1">
-      <c r="A9" s="30" t="inlineStr">
+      <c r="A9" s="31" t="inlineStr">
         <is>
           <t>Q2 2026
 Phase 1 Start</t>
         </is>
       </c>
-      <c r="B9" s="12" t="inlineStr">
-        <is>
-          <t>Startschuss · 10 Leitbetriebe · 100 Betriebe Q4</t>
-        </is>
-      </c>
-      <c r="C9" s="31" t="inlineStr">
-        <is>
-          <t>Partnerschaftsvertrag · Budget-Freigabe · MRV-Software go-live</t>
-        </is>
-      </c>
-      <c r="D9" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E9" s="32" t="inlineStr">
+      <c r="B9" s="8" t="inlineStr">
+        <is>
+          <t>Startschuss · 10 Leitbetriebe · Budget-Freigabe</t>
+        </is>
+      </c>
+      <c r="C9" s="32" t="inlineStr">
+        <is>
+          <t>Partnerschaftsvertrag · Schnittstellenentwicklung · MRV-Software go-live</t>
+        </is>
+      </c>
+      <c r="D9" s="33" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E9" s="33" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
     </row>
     <row r="10" ht="34" customHeight="1">
-      <c r="A10" s="33" t="inlineStr">
+      <c r="A10" s="34" t="inlineStr">
+        <is>
+          <t>Q3–Q4 2026
+Onboarding-Kampagne</t>
+        </is>
+      </c>
+      <c r="B10" s="10" t="inlineStr">
+        <is>
+          <t>~100 neue Betriebe · Verra-Dossier aufbereitet</t>
+        </is>
+      </c>
+      <c r="C10" s="35" t="inlineStr">
+        <is>
+          <t>Hofgespräche · Baseline, Bodenproben &amp; Laboranalysen · Hist. Daten</t>
+        </is>
+      </c>
+      <c r="D10" s="36" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E10" s="36" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="34" customHeight="1">
+      <c r="A11" s="31" t="inlineStr">
         <is>
           <t>Q1 2027
 Verra-Einreichung</t>
         </is>
       </c>
-      <c r="B10" s="14" t="inlineStr">
+      <c r="B11" s="8" t="inlineStr">
         <is>
           <t>100 Betriebe aktiv · 10.000 ha · PDD eingereicht</t>
         </is>
       </c>
-      <c r="C10" s="34" t="inlineStr">
-        <is>
-          <t>2. Beprobungsrunde · VVB gestartet · BE Trading-Netzwerk aufgebaut</t>
-        </is>
-      </c>
-      <c r="D10" s="35" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E10" s="35" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" ht="34" customHeight="1">
-      <c r="A11" s="45" t="inlineStr">
+      <c r="C11" s="32" t="inlineStr">
+        <is>
+          <t>2. Beprobungsrunde · VVB gestartet · BE Trading-Vermarktungsstruktur</t>
+        </is>
+      </c>
+      <c r="D11" s="33" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E11" s="33" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="34" customHeight="1">
+      <c r="A12" s="47" t="inlineStr">
         <is>
           <t>Q2/Q3 2027
 🎯 TRANCHE 1</t>
         </is>
       </c>
-      <c r="B11" s="46" t="inlineStr">
+      <c r="B12" s="48" t="inlineStr">
         <is>
           <t>Erster Zertifikatsverkauf · 5.000 t</t>
         </is>
       </c>
-      <c r="C11" s="47" t="inlineStr">
-        <is>
-          <t>Verra VCU-Issuance · CORSIA-fähig · Burgenland als Referenz</t>
-        </is>
-      </c>
-      <c r="D11" s="48" t="n">
+      <c r="C12" s="49" t="inlineStr">
+        <is>
+          <t>Verra VCU-Issuance T1 · CORSIA-fähig · Burgenland als Referenzmodell</t>
+        </is>
+      </c>
+      <c r="D12" s="50" t="n">
         <v>5000</v>
       </c>
-      <c r="E11" s="49" t="n">
+      <c r="E12" s="51" t="n">
         <v>430000</v>
       </c>
     </row>
-    <row r="12" ht="34" customHeight="1">
-      <c r="A12" s="33" t="inlineStr">
+    <row r="13" ht="34" customHeight="1">
+      <c r="A13" s="31" t="inlineStr">
         <is>
           <t>2028
-+50% Enrollment</t>
-        </is>
-      </c>
-      <c r="B12" s="14" t="inlineStr">
-        <is>
-          <t>300 Betriebe · ~30.000 ha</t>
-        </is>
-      </c>
-      <c r="C12" s="34" t="inlineStr">
-        <is>
-          <t>360K-Zusatz: Onboarding-Skalierung · Enrollment +50% gegenüber 2027</t>
-        </is>
-      </c>
-      <c r="D12" s="35" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E12" s="35" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-    </row>
-    <row r="13" ht="34" customHeight="1">
-      <c r="A13" s="45" t="inlineStr">
+Skalierung</t>
+        </is>
+      </c>
+      <c r="B13" s="8" t="inlineStr">
+        <is>
+          <t>500 Betriebe aktiv · 50.000+ ha</t>
+        </is>
+      </c>
+      <c r="C13" s="32" t="inlineStr">
+        <is>
+          <t>360K-Onboarding-Push · CORSIA-Verträge · freiwilliger Markt · Expansion gestartet</t>
+        </is>
+      </c>
+      <c r="D13" s="33" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E13" s="33" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="34" customHeight="1">
+      <c r="A14" s="47" t="inlineStr">
         <is>
           <t>2029
 🎯 TRANCHE 2</t>
         </is>
       </c>
-      <c r="B13" s="46" t="inlineStr">
-        <is>
-          <t>25.000 t · Österreich-Ausbau</t>
-        </is>
-      </c>
-      <c r="C13" s="47" t="inlineStr">
-        <is>
-          <t>Verra VCU-Issuance T2 · CORSIA-Verträge · freiwilliger Markt</t>
-        </is>
-      </c>
-      <c r="D13" s="48" t="n">
+      <c r="B14" s="48" t="inlineStr">
+        <is>
+          <t>25.000 t · 750 Betriebe · AT-Referenzmodell</t>
+        </is>
+      </c>
+      <c r="C14" s="49" t="inlineStr">
+        <is>
+          <t>Verra VCU-Issuance T2 · 2,5–3,75 Mio € Umsatz BE Trading</t>
+        </is>
+      </c>
+      <c r="D14" s="50" t="n">
         <v>25000</v>
       </c>
-      <c r="E13" s="49" t="n">
+      <c r="E14" s="51" t="n">
         <v>2150000</v>
       </c>
     </row>
-    <row r="14" ht="34" customHeight="1">
-      <c r="A14" s="33" t="inlineStr">
+    <row r="15" ht="34" customHeight="1">
+      <c r="A15" s="31" t="inlineStr">
         <is>
           <t>Ab 2030
 Jährliches Ernten</t>
         </is>
       </c>
-      <c r="B14" s="14" t="inlineStr">
-        <is>
-          <t>~12.000 t/yr</t>
-        </is>
-      </c>
-      <c r="C14" s="34" t="inlineStr">
-        <is>
-          <t>Stabiler Monitoring-Zyklus · jährliche Credit-Ernte</t>
-        </is>
-      </c>
-      <c r="D14" s="35" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E14" s="35" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-    </row>
-    <row r="16" ht="26" customHeight="1">
-      <c r="A16" s="44" t="inlineStr">
-        <is>
-          <t>BE Trading Marge — T1 + T2 (Einkauf @ 86€/t)</t>
-        </is>
-      </c>
-    </row>
-    <row r="17" ht="20" customHeight="1">
-      <c r="A17" s="29" t="inlineStr">
+      <c r="B15" s="8" t="inlineStr">
+        <is>
+          <t>~12.000 t/yr · stabiles Portfolio</t>
+        </is>
+      </c>
+      <c r="C15" s="32" t="inlineStr">
+        <is>
+          <t>Jährlicher Monitoring-Zyklus · wachsende Credit-Ernte</t>
+        </is>
+      </c>
+      <c r="D15" s="33" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E15" s="33" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="26" customHeight="1">
+      <c r="A17" s="46" t="inlineStr">
+        <is>
+          <t>BE Trading Marge — Tranche 1 + Tranche 2 (Einkauf @ 86 €/t)</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="20" customHeight="1">
+      <c r="A18" s="30" t="inlineStr">
         <is>
           <t>Verkaufspreis</t>
         </is>
       </c>
-      <c r="B17" s="29" t="inlineStr">
+      <c r="B18" s="30" t="inlineStr">
         <is>
           <t>T1 Einkauf</t>
         </is>
       </c>
-      <c r="C17" s="29" t="inlineStr">
+      <c r="C18" s="30" t="inlineStr">
         <is>
           <t>T1 Marge</t>
         </is>
       </c>
-      <c r="D17" s="29" t="inlineStr">
+      <c r="D18" s="30" t="inlineStr">
         <is>
           <t>T2 Einkauf</t>
         </is>
       </c>
-      <c r="E17" s="29" t="inlineStr">
+      <c r="E18" s="30" t="inlineStr">
         <is>
           <t>T2 Marge</t>
         </is>
       </c>
     </row>
-    <row r="18" ht="22" customHeight="1">
-      <c r="A18" s="9" t="inlineStr">
+    <row r="19" ht="22" customHeight="1">
+      <c r="A19" s="18" t="inlineStr">
         <is>
           <t>@ 100 €/t</t>
-        </is>
-      </c>
-      <c r="B18" s="50" t="n">
-        <v>430000</v>
-      </c>
-      <c r="C18" s="51" t="n">
-        <v>70000</v>
-      </c>
-      <c r="D18" s="50" t="n">
-        <v>2150000</v>
-      </c>
-      <c r="E18" s="51" t="n">
-        <v>350000</v>
-      </c>
-    </row>
-    <row r="19" ht="22" customHeight="1">
-      <c r="A19" s="11" t="inlineStr">
-        <is>
-          <t>@ 125 €/t</t>
         </is>
       </c>
       <c r="B19" s="52" t="n">
         <v>430000</v>
       </c>
       <c r="C19" s="53" t="n">
-        <v>195000</v>
+        <v>70000</v>
       </c>
       <c r="D19" s="52" t="n">
         <v>2150000</v>
       </c>
       <c r="E19" s="53" t="n">
+        <v>350000</v>
+      </c>
+    </row>
+    <row r="20" ht="22" customHeight="1">
+      <c r="A20" s="15" t="inlineStr">
+        <is>
+          <t>@ 125 €/t</t>
+        </is>
+      </c>
+      <c r="B20" s="54" t="n">
+        <v>430000</v>
+      </c>
+      <c r="C20" s="55" t="n">
+        <v>195000</v>
+      </c>
+      <c r="D20" s="54" t="n">
+        <v>2150000</v>
+      </c>
+      <c r="E20" s="55" t="n">
         <v>975000</v>
       </c>
     </row>
-    <row r="20" ht="22" customHeight="1">
-      <c r="A20" s="9" t="inlineStr">
+    <row r="21" ht="22" customHeight="1">
+      <c r="A21" s="18" t="inlineStr">
         <is>
           <t>@ 150 €/t</t>
         </is>
       </c>
-      <c r="B20" s="50" t="n">
+      <c r="B21" s="52" t="n">
         <v>430000</v>
       </c>
-      <c r="C20" s="51" t="n">
+      <c r="C21" s="53" t="n">
         <v>320000</v>
       </c>
-      <c r="D20" s="50" t="n">
+      <c r="D21" s="52" t="n">
         <v>2150000</v>
       </c>
-      <c r="E20" s="51" t="n">
+      <c r="E21" s="53" t="n">
         <v>1600000</v>
       </c>
     </row>
-    <row r="21" ht="30" customHeight="1">
-      <c r="A21" s="54" t="inlineStr">
+    <row r="22" ht="30" customHeight="1">
+      <c r="A22" s="56" t="inlineStr">
         <is>
           <t>KUMULIERT T1+T2 @ 150€</t>
         </is>
       </c>
-      <c r="B21" s="55" t="n">
+      <c r="B22" s="57" t="n">
         <v>2580000</v>
       </c>
-      <c r="C21" s="56" t="inlineStr">
+      <c r="C22" s="58" t="inlineStr">
         <is>
           <t>Kumulierte Marge für BE Trading: 1,920,000 €</t>
         </is>
@@ -2029,10 +2186,10 @@
   </sheetData>
   <mergeCells count="5">
     <mergeCell ref="A2:E2"/>
-    <mergeCell ref="A16:E16"/>
     <mergeCell ref="A7:E7"/>
+    <mergeCell ref="C22:E22"/>
     <mergeCell ref="A1:E1"/>
-    <mergeCell ref="C21:E21"/>
+    <mergeCell ref="A17:E17"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -2044,388 +2201,416 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E22"/>
+  <dimension ref="A1:E23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
     <col width="32" customWidth="1" min="2" max="2"/>
-    <col width="38" customWidth="1" min="3" max="3"/>
+    <col width="40" customWidth="1" min="3" max="3"/>
     <col width="18" customWidth="1" min="4" max="4"/>
     <col width="18" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1" ht="34" customHeight="1">
-      <c r="A1" s="57" t="inlineStr">
+      <c r="A1" s="59" t="inlineStr">
         <is>
           <t>Ground UP × BE  ·  1M AT-Exklusivität</t>
         </is>
       </c>
     </row>
     <row r="2" ht="18" customHeight="1">
-      <c r="A2" s="58" t="inlineStr">
-        <is>
-          <t>AT-Markt-Exklusivität · +100% Enrollment-Wachstum 2029</t>
+      <c r="A2" s="60" t="inlineStr">
+        <is>
+          <t>AT-Markt-Exklusivität · 2× Skalierung der 500K-Basis</t>
         </is>
       </c>
     </row>
     <row r="3" ht="28" customHeight="1">
-      <c r="A3" s="59" t="inlineStr">
-        <is>
-          <t>⭐  Dieses Paket beinhaltet die Markt-Exklusivität für Burgenland Energie im österreichischen Carbon-Farming-Markt.</t>
+      <c r="A3" s="61" t="inlineStr">
+        <is>
+          <t>⭐  Dieses Paket beinhaltet die Markt-Exklusivität für Burgenland Energie im gesamten österreichischen Carbon-Farming-Markt.</t>
         </is>
       </c>
     </row>
     <row r="5" ht="20" customHeight="1">
-      <c r="A5" s="6" t="inlineStr">
+      <c r="A5" s="62" t="inlineStr">
         <is>
           <t>Gesamt-Investment</t>
         </is>
       </c>
-      <c r="B5" s="6" t="inlineStr">
+      <c r="B5" s="62" t="inlineStr">
         <is>
           <t>Tranche 1</t>
         </is>
       </c>
-      <c r="C5" s="6" t="inlineStr">
+      <c r="C5" s="62" t="inlineStr">
         <is>
           <t>Tranche 2</t>
         </is>
       </c>
-      <c r="D5" s="6" t="inlineStr">
+      <c r="D5" s="62" t="inlineStr">
         <is>
           <t>Betriebe 2028</t>
         </is>
       </c>
-      <c r="E5" s="6" t="inlineStr">
+      <c r="E5" s="62" t="inlineStr">
         <is>
           <t>Hektar 2028</t>
         </is>
       </c>
     </row>
-    <row r="6" ht="32" customHeight="1">
-      <c r="A6" s="60" t="inlineStr">
-        <is>
-          <t>1,000,000 €</t>
-        </is>
-      </c>
-      <c r="B6" s="60" t="inlineStr">
+    <row r="6" ht="34" customHeight="1">
+      <c r="A6" s="63" t="inlineStr">
+        <is>
+          <t>1.000.000 €</t>
+        </is>
+      </c>
+      <c r="B6" s="63" t="inlineStr">
         <is>
           <t>5.000 t
 (Q2/Q3 2027)</t>
         </is>
       </c>
-      <c r="C6" s="60" t="inlineStr">
-        <is>
-          <t>50,000 t
+      <c r="C6" s="63" t="inlineStr">
+        <is>
+          <t>50.000 t
 (2029)</t>
         </is>
       </c>
-      <c r="D6" s="60" t="inlineStr">
-        <is>
-          <t>500</t>
-        </is>
-      </c>
-      <c r="E6" s="60" t="inlineStr">
-        <is>
-          <t>60,000 ha</t>
+      <c r="D6" s="63" t="inlineStr">
+        <is>
+          <t>1.000</t>
+        </is>
+      </c>
+      <c r="E6" s="63" t="inlineStr">
+        <is>
+          <t>100.000+ ha</t>
         </is>
       </c>
     </row>
     <row r="8" ht="26" customHeight="1">
-      <c r="A8" s="61" t="inlineStr">
-        <is>
-          <t>Meilensteinplan — aligned mit Pitch Burgenland Energie (2026–2030+)</t>
+      <c r="A8" s="64" t="inlineStr">
+        <is>
+          <t>Meilensteinplan — Ground UP × Burgenland Energie (2026–2030+)</t>
         </is>
       </c>
     </row>
     <row r="9" ht="22" customHeight="1">
-      <c r="A9" s="29" t="inlineStr">
+      <c r="A9" s="30" t="inlineStr">
         <is>
           <t>Phase</t>
         </is>
       </c>
-      <c r="B9" s="29" t="inlineStr">
+      <c r="B9" s="30" t="inlineStr">
         <is>
           <t>Milestone</t>
         </is>
       </c>
-      <c r="C9" s="29" t="inlineStr">
+      <c r="C9" s="30" t="inlineStr">
         <is>
           <t>Aktivitäten &amp; Deliverables</t>
         </is>
       </c>
-      <c r="D9" s="29" t="inlineStr">
+      <c r="D9" s="30" t="inlineStr">
         <is>
           <t>Tonnen</t>
         </is>
       </c>
-      <c r="E9" s="29" t="inlineStr">
+      <c r="E9" s="30" t="inlineStr">
         <is>
           <t>Erlös BE @ 86€</t>
         </is>
       </c>
     </row>
     <row r="10" ht="34" customHeight="1">
-      <c r="A10" s="30" t="inlineStr">
+      <c r="A10" s="31" t="inlineStr">
         <is>
           <t>Q2 2026
 Phase 1 Start</t>
         </is>
       </c>
-      <c r="B10" s="12" t="inlineStr">
+      <c r="B10" s="8" t="inlineStr">
         <is>
           <t>Startschuss · AT-Exklusivitätsvertrag · 10 Leitbetriebe</t>
         </is>
       </c>
-      <c r="C10" s="31" t="inlineStr">
+      <c r="C10" s="32" t="inlineStr">
         <is>
           <t>Partnerschaftsvertrag inkl. AT-Markt-Exklusivität · MRV-Software go-live</t>
         </is>
       </c>
-      <c r="D10" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E10" s="32" t="inlineStr">
+      <c r="D10" s="33" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E10" s="33" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
     </row>
     <row r="11" ht="34" customHeight="1">
-      <c r="A11" s="33" t="inlineStr">
+      <c r="A11" s="34" t="inlineStr">
+        <is>
+          <t>Q3–Q4 2026
+Onboarding-Kampagne</t>
+        </is>
+      </c>
+      <c r="B11" s="10" t="inlineStr">
+        <is>
+          <t>~100 neue Betriebe · Verra-Dossier aufbereitet</t>
+        </is>
+      </c>
+      <c r="C11" s="35" t="inlineStr">
+        <is>
+          <t>Hofgespräche · Baseline, Bodenproben &amp; Laboranalysen · Hist. Daten</t>
+        </is>
+      </c>
+      <c r="D11" s="36" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E11" s="36" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="34" customHeight="1">
+      <c r="A12" s="31" t="inlineStr">
         <is>
           <t>Q1 2027
 Verra-Einreichung</t>
         </is>
       </c>
-      <c r="B11" s="14" t="inlineStr">
+      <c r="B12" s="8" t="inlineStr">
         <is>
           <t>100 Betriebe aktiv · 10.000 ha · PDD eingereicht</t>
         </is>
       </c>
-      <c r="C11" s="34" t="inlineStr">
+      <c r="C12" s="32" t="inlineStr">
         <is>
           <t>2. Beprobungsrunde · VVB gestartet · AT-weites Rollout startet</t>
         </is>
       </c>
-      <c r="D11" s="35" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E11" s="35" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-    </row>
-    <row r="12" ht="34" customHeight="1">
-      <c r="A12" s="62" t="inlineStr">
+      <c r="D12" s="33" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E12" s="33" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="34" customHeight="1">
+      <c r="A13" s="65" t="inlineStr">
         <is>
           <t>Q2/Q3 2027
 🎯 TRANCHE 1</t>
         </is>
       </c>
-      <c r="B12" s="63" t="inlineStr">
+      <c r="B13" s="66" t="inlineStr">
         <is>
           <t>Erster Zertifikatsverkauf · 5.000 t</t>
         </is>
       </c>
-      <c r="C12" s="64" t="inlineStr">
-        <is>
-          <t>Verra VCU-Issuance · CORSIA-fähig · BE als exklusiver AT-Partner</t>
-        </is>
-      </c>
-      <c r="D12" s="65" t="n">
+      <c r="C13" s="67" t="inlineStr">
+        <is>
+          <t>Verra VCU-Issuance T1 · CORSIA-fähig · BE als exklusiver AT-Partner</t>
+        </is>
+      </c>
+      <c r="D13" s="68" t="n">
         <v>5000</v>
       </c>
-      <c r="E12" s="66" t="n">
+      <c r="E13" s="69" t="n">
         <v>430000</v>
       </c>
     </row>
-    <row r="13" ht="34" customHeight="1">
-      <c r="A13" s="33" t="inlineStr">
+    <row r="14" ht="34" customHeight="1">
+      <c r="A14" s="31" t="inlineStr">
         <is>
           <t>2028
-+100% Enrollment</t>
-        </is>
-      </c>
-      <c r="B13" s="14" t="inlineStr">
-        <is>
-          <t>500 Betriebe · ~60.000 ha</t>
-        </is>
-      </c>
-      <c r="C13" s="34" t="inlineStr">
-        <is>
-          <t>860K-Zusatz: Massives AT-Onboarding · Enrollment verdoppelt sich 2029</t>
-        </is>
-      </c>
-      <c r="D13" s="35" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E13" s="35" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-    </row>
-    <row r="14" ht="34" customHeight="1">
-      <c r="A14" s="62" t="inlineStr">
+AT-Rollout</t>
+        </is>
+      </c>
+      <c r="B14" s="8" t="inlineStr">
+        <is>
+          <t>1.000 Betriebe aktiv · 100.000+ ha</t>
+        </is>
+      </c>
+      <c r="C14" s="32" t="inlineStr">
+        <is>
+          <t>860K-Push: Burgenland + AT-Expansion · CORSIA-Verträge · EU-Markt</t>
+        </is>
+      </c>
+      <c r="D14" s="33" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E14" s="33" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="34" customHeight="1">
+      <c r="A15" s="65" t="inlineStr">
         <is>
           <t>2029
 🎯 TRANCHE 2</t>
         </is>
       </c>
-      <c r="B14" s="63" t="inlineStr">
-        <is>
-          <t>50.000 t · AT als EU-Referenzmodell</t>
-        </is>
-      </c>
-      <c r="C14" s="64" t="inlineStr">
-        <is>
-          <t>Verra VCU-Issuance T2 · CORSIA-Verträge · BE einziger AT-Anbieter</t>
-        </is>
-      </c>
-      <c r="D14" s="65" t="n">
+      <c r="B15" s="66" t="inlineStr">
+        <is>
+          <t>50.000 t · 1.500 Betriebe · EU-Referenzmodell</t>
+        </is>
+      </c>
+      <c r="C15" s="67" t="inlineStr">
+        <is>
+          <t>Verra VCU-Issuance T2 · 5–7,5 Mio € Umsatz BE Trading · AT-Marktführer</t>
+        </is>
+      </c>
+      <c r="D15" s="68" t="n">
         <v>50000</v>
       </c>
-      <c r="E14" s="66" t="n">
+      <c r="E15" s="69" t="n">
         <v>4300000</v>
       </c>
     </row>
-    <row r="15" ht="34" customHeight="1">
-      <c r="A15" s="33" t="inlineStr">
+    <row r="16" ht="34" customHeight="1">
+      <c r="A16" s="31" t="inlineStr">
         <is>
           <t>Ab 2030
 Jährliches Ernten</t>
         </is>
       </c>
-      <c r="B15" s="14" t="inlineStr">
-        <is>
-          <t>~32.000 t/yr</t>
-        </is>
-      </c>
-      <c r="C15" s="34" t="inlineStr">
-        <is>
-          <t>Vollständig etabliertes AT-Portfolio · jährliche Credit-Ernte · EU-Expansion</t>
-        </is>
-      </c>
-      <c r="D15" s="35" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E15" s="35" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-    </row>
-    <row r="17" ht="26" customHeight="1">
-      <c r="A17" s="61" t="inlineStr">
-        <is>
-          <t>BE Trading Marge — T1 + T2 (Einkauf @ 86€/t)</t>
-        </is>
-      </c>
-    </row>
-    <row r="18" ht="20" customHeight="1">
-      <c r="A18" s="29" t="inlineStr">
+      <c r="B16" s="8" t="inlineStr">
+        <is>
+          <t>~32.000 t/yr · AT-weites Portfolio</t>
+        </is>
+      </c>
+      <c r="C16" s="32" t="inlineStr">
+        <is>
+          <t>Jährlicher Monitoring-Zyklus · BE einziger AT-Anbieter</t>
+        </is>
+      </c>
+      <c r="D16" s="33" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E16" s="33" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="26" customHeight="1">
+      <c r="A18" s="64" t="inlineStr">
+        <is>
+          <t>BE Trading Marge — Tranche 1 + Tranche 2 (Einkauf @ 86 €/t)</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="20" customHeight="1">
+      <c r="A19" s="30" t="inlineStr">
         <is>
           <t>Verkaufspreis</t>
         </is>
       </c>
-      <c r="B18" s="29" t="inlineStr">
+      <c r="B19" s="30" t="inlineStr">
         <is>
           <t>T1 Einkauf</t>
         </is>
       </c>
-      <c r="C18" s="29" t="inlineStr">
+      <c r="C19" s="30" t="inlineStr">
         <is>
           <t>T1 Marge</t>
         </is>
       </c>
-      <c r="D18" s="29" t="inlineStr">
+      <c r="D19" s="30" t="inlineStr">
         <is>
           <t>T2 Einkauf</t>
         </is>
       </c>
-      <c r="E18" s="29" t="inlineStr">
+      <c r="E19" s="30" t="inlineStr">
         <is>
           <t>T2 Marge</t>
         </is>
       </c>
     </row>
-    <row r="19" ht="22" customHeight="1">
-      <c r="A19" s="9" t="inlineStr">
+    <row r="20" ht="22" customHeight="1">
+      <c r="A20" s="18" t="inlineStr">
         <is>
           <t>@ 100 €/t</t>
-        </is>
-      </c>
-      <c r="B19" s="50" t="n">
-        <v>430000</v>
-      </c>
-      <c r="C19" s="51" t="n">
-        <v>70000</v>
-      </c>
-      <c r="D19" s="50" t="n">
-        <v>4300000</v>
-      </c>
-      <c r="E19" s="51" t="n">
-        <v>700000</v>
-      </c>
-    </row>
-    <row r="20" ht="22" customHeight="1">
-      <c r="A20" s="11" t="inlineStr">
-        <is>
-          <t>@ 125 €/t</t>
         </is>
       </c>
       <c r="B20" s="52" t="n">
         <v>430000</v>
       </c>
       <c r="C20" s="53" t="n">
-        <v>195000</v>
+        <v>70000</v>
       </c>
       <c r="D20" s="52" t="n">
         <v>4300000</v>
       </c>
       <c r="E20" s="53" t="n">
+        <v>700000</v>
+      </c>
+    </row>
+    <row r="21" ht="22" customHeight="1">
+      <c r="A21" s="15" t="inlineStr">
+        <is>
+          <t>@ 125 €/t</t>
+        </is>
+      </c>
+      <c r="B21" s="54" t="n">
+        <v>430000</v>
+      </c>
+      <c r="C21" s="55" t="n">
+        <v>195000</v>
+      </c>
+      <c r="D21" s="54" t="n">
+        <v>4300000</v>
+      </c>
+      <c r="E21" s="55" t="n">
         <v>1950000</v>
       </c>
     </row>
-    <row r="21" ht="22" customHeight="1">
-      <c r="A21" s="9" t="inlineStr">
+    <row r="22" ht="22" customHeight="1">
+      <c r="A22" s="18" t="inlineStr">
         <is>
           <t>@ 150 €/t</t>
         </is>
       </c>
-      <c r="B21" s="50" t="n">
+      <c r="B22" s="52" t="n">
         <v>430000</v>
       </c>
-      <c r="C21" s="51" t="n">
+      <c r="C22" s="53" t="n">
         <v>320000</v>
       </c>
-      <c r="D21" s="50" t="n">
+      <c r="D22" s="52" t="n">
         <v>4300000</v>
       </c>
-      <c r="E21" s="51" t="n">
+      <c r="E22" s="53" t="n">
         <v>3200000</v>
       </c>
     </row>
-    <row r="22" ht="30" customHeight="1">
-      <c r="A22" s="54" t="inlineStr">
+    <row r="23" ht="30" customHeight="1">
+      <c r="A23" s="56" t="inlineStr">
         <is>
           <t>KUMULIERT T1+T2 @ 150€</t>
         </is>
       </c>
-      <c r="B22" s="55" t="n">
+      <c r="B23" s="57" t="n">
         <v>4730000</v>
       </c>
-      <c r="C22" s="56" t="inlineStr">
+      <c r="C23" s="58" t="inlineStr">
         <is>
           <t>Kumulierte Marge für BE Trading: 3,520,000 €</t>
         </is>
@@ -2434,10 +2619,10 @@
   </sheetData>
   <mergeCells count="6">
     <mergeCell ref="A2:E2"/>
-    <mergeCell ref="C22:E22"/>
+    <mergeCell ref="C23:E23"/>
     <mergeCell ref="A1:E1"/>
     <mergeCell ref="A8:E8"/>
-    <mergeCell ref="A17:E17"/>
+    <mergeCell ref="A18:E18"/>
     <mergeCell ref="A3:E3"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -2450,233 +2635,221 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B20"/>
+  <dimension ref="A1:B19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
-    <col width="70" customWidth="1" min="2" max="2"/>
+    <col width="72" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
     <row r="1" ht="32" customHeight="1">
-      <c r="A1" s="67" t="inlineStr">
+      <c r="A1" s="70" t="inlineStr">
         <is>
           <t>Annahmen &amp; Methodik — Ground UP × Burgenland Energie</t>
         </is>
       </c>
     </row>
     <row r="3" ht="22" customHeight="1">
-      <c r="A3" s="8" t="inlineStr">
+      <c r="A3" s="17" t="inlineStr">
         <is>
           <t>Standard</t>
         </is>
       </c>
-      <c r="B3" s="12" t="inlineStr">
+      <c r="B3" s="8" t="inlineStr">
         <is>
           <t>Verra VM0042 v2.2 + VT0014 v1.0 (Soil Organic Carbon)</t>
         </is>
       </c>
     </row>
     <row r="4" ht="22" customHeight="1">
-      <c r="A4" s="10" t="inlineStr">
+      <c r="A4" s="14" t="inlineStr">
         <is>
           <t>SOC-Steigerung</t>
         </is>
       </c>
-      <c r="B4" s="14" t="inlineStr">
+      <c r="B4" s="10" t="inlineStr">
         <is>
           <t>2,5 t CO₂e/ha/yr (konservativ, VM0042-konform)</t>
         </is>
       </c>
     </row>
     <row r="5" ht="22" customHeight="1">
-      <c r="A5" s="8" t="inlineStr">
+      <c r="A5" s="17" t="inlineStr">
         <is>
           <t>Buffer Pool</t>
         </is>
       </c>
-      <c r="B5" s="12" t="inlineStr">
+      <c r="B5" s="8" t="inlineStr">
         <is>
           <t>25 % (12,5 % Verra Puffer + 12,5 % Ground UP Reserve)</t>
         </is>
       </c>
     </row>
     <row r="6" ht="22" customHeight="1">
-      <c r="A6" s="10" t="inlineStr">
+      <c r="A6" s="14" t="inlineStr">
         <is>
           <t>Unsicherheit</t>
         </is>
       </c>
-      <c r="B6" s="14" t="inlineStr">
+      <c r="B6" s="10" t="inlineStr">
         <is>
           <t>15 % (formelbasiert VM0042)</t>
         </is>
       </c>
     </row>
     <row r="7" ht="22" customHeight="1">
-      <c r="A7" s="8" t="inlineStr">
+      <c r="A7" s="17" t="inlineStr">
         <is>
           <t>Netto-Ertrag</t>
         </is>
       </c>
-      <c r="B7" s="12" t="inlineStr">
+      <c r="B7" s="8" t="inlineStr">
         <is>
           <t>~1,87 t CO₂e/ha/yr netto (nach Buffer + Unsicherheit)</t>
         </is>
       </c>
     </row>
     <row r="8" ht="22" customHeight="1">
-      <c r="A8" s="10" t="inlineStr">
+      <c r="A8" s="14" t="inlineStr">
         <is>
           <t>Kreditpreis an BE</t>
         </is>
       </c>
-      <c r="B8" s="14" t="inlineStr">
+      <c r="B8" s="10" t="inlineStr">
         <is>
           <t>86 €/t (vertraglich vereinbart)</t>
         </is>
       </c>
     </row>
     <row r="9" ht="22" customHeight="1">
-      <c r="A9" s="8" t="inlineStr">
+      <c r="A9" s="17" t="inlineStr">
         <is>
           <t>BE Break-even</t>
         </is>
       </c>
-      <c r="B9" s="12" t="inlineStr">
+      <c r="B9" s="8" t="inlineStr">
         <is>
           <t>100 €/t Weiterverkauf</t>
         </is>
       </c>
     </row>
     <row r="10" ht="22" customHeight="1">
-      <c r="A10" s="10" t="inlineStr">
+      <c r="A10" s="14" t="inlineStr">
         <is>
           <t>BE Zielpreis</t>
         </is>
       </c>
-      <c r="B10" s="14" t="inlineStr">
+      <c r="B10" s="10" t="inlineStr">
         <is>
           <t>150 €/t (CORSIA-Markt, BE Trading)</t>
         </is>
       </c>
     </row>
     <row r="11" ht="22" customHeight="1">
-      <c r="A11" s="8" t="inlineStr">
+      <c r="A11" s="17" t="inlineStr">
+        <is>
+          <t>Pitch-Basis</t>
+        </is>
+      </c>
+      <c r="B11" s="8" t="inlineStr">
+        <is>
+          <t>500K-Szenario entspricht exakt den Zahlen im Pitch (500 Betriebe 2028 / 25.000 t T2 2029 / 750 Betriebe)</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="22" customHeight="1">
+      <c r="A12" s="14" t="inlineStr">
+        <is>
+          <t>1M-Skalierung</t>
+        </is>
+      </c>
+      <c r="B12" s="10" t="inlineStr">
+        <is>
+          <t>1M = 2× die 500K-Basis (1.000 Betriebe 2028 / 50.000 t T2 / 1.500 Betriebe 2029 / 150.000+ ha)</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="22" customHeight="1">
+      <c r="A13" s="17" t="inlineStr">
+        <is>
+          <t>AT-Exklusivität</t>
+        </is>
+      </c>
+      <c r="B13" s="8" t="inlineStr">
+        <is>
+          <t>1M-Investment beinhaltet Markt-Exklusivität für BE im österreichischen Carbon-Farming-Markt</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="22" customHeight="1">
+      <c r="A14" s="14" t="inlineStr">
         <is>
           <t>Tranche 1</t>
         </is>
       </c>
-      <c r="B11" s="12" t="inlineStr">
-        <is>
-          <t>5.000 t netto — historische Daten aus bestehenden Pilotbetrieben (alle Szenarien)</t>
-        </is>
-      </c>
-    </row>
-    <row r="12" ht="22" customHeight="1">
-      <c r="A12" s="10" t="inlineStr">
+      <c r="B14" s="10" t="inlineStr">
+        <is>
+          <t>5.000 t netto — historische Daten aus bestehenden Pilotbetrieben</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="22" customHeight="1">
+      <c r="A15" s="17" t="inlineStr">
         <is>
           <t>Tranche-Rhythmus</t>
         </is>
       </c>
-      <c r="B12" s="14" t="inlineStr">
-        <is>
-          <t>Alle 3–5 Jahre; intensive Portfolio-Aufbauphase vor jeder Tranche</t>
-        </is>
-      </c>
-    </row>
-    <row r="13" ht="22" customHeight="1">
-      <c r="A13" s="8" t="inlineStr">
-        <is>
-          <t>Enrollment-Wachstum</t>
-        </is>
-      </c>
-      <c r="B13" s="12" t="inlineStr">
-        <is>
-          <t>Enrollment = Baseline, Bodenproben, Laboranalyse und historische Datenaufbereitung je Betrieb</t>
-        </is>
-      </c>
-    </row>
-    <row r="14" ht="22" customHeight="1">
-      <c r="A14" s="10" t="inlineStr">
-        <is>
-          <t>500K: +50%</t>
-        </is>
-      </c>
-      <c r="B14" s="14" t="inlineStr">
-        <is>
-          <t>Enrollment-Wachstum 2029 +50% gegenüber 2027-Basis → Tranche 2: 25.000 t</t>
-        </is>
-      </c>
-    </row>
-    <row r="15" ht="22" customHeight="1">
-      <c r="A15" s="8" t="inlineStr">
-        <is>
-          <t>1M: +100%</t>
-        </is>
-      </c>
-      <c r="B15" s="12" t="inlineStr">
-        <is>
-          <t>Enrollment-Wachstum 2029 +100% gegenüber 2027-Basis → Tranche 2: 50.000 t</t>
+      <c r="B15" s="8" t="inlineStr">
+        <is>
+          <t>Alle 3–5 Jahre; Portfolio-Aufbauphase vor jeder Tranche</t>
         </is>
       </c>
     </row>
     <row r="16" ht="22" customHeight="1">
-      <c r="A16" s="10" t="inlineStr">
-        <is>
-          <t>AT-Exklusivität</t>
-        </is>
-      </c>
-      <c r="B16" s="14" t="inlineStr">
-        <is>
-          <t>1M-Investment beinhaltet Markt-Exklusivität für BE im österreichischen Carbon-Farming-Markt</t>
+      <c r="A16" s="14" t="inlineStr">
+        <is>
+          <t>Enrollment</t>
+        </is>
+      </c>
+      <c r="B16" s="10" t="inlineStr">
+        <is>
+          <t>Baseline, initiale Bodenproben, Laboranalyse und historische Datenaufbereitung je Betrieb</t>
         </is>
       </c>
     </row>
     <row r="17" ht="22" customHeight="1">
-      <c r="A17" s="8" t="inlineStr">
+      <c r="A17" s="17" t="inlineStr">
         <is>
           <t>CORSIA</t>
         </is>
       </c>
-      <c r="B17" s="12" t="inlineStr">
+      <c r="B17" s="8" t="inlineStr">
         <is>
           <t>Phase II ab 2027 — wachsende Nachfrage Luftfahrt EU · Preistreiber 100–150+ €/t</t>
         </is>
       </c>
     </row>
     <row r="18" ht="22" customHeight="1">
-      <c r="A18" s="10" t="inlineStr">
+      <c r="A18" s="14" t="inlineStr">
         <is>
           <t>MRV-System</t>
         </is>
       </c>
-      <c r="B18" s="14" t="inlineStr">
+      <c r="B18" s="10" t="inlineStr">
         <is>
           <t>SOMA — KI-Bodenmodell EU-nativ · Sentinel-2 + ERA5-Land + LUCAS Soil DB + Laborproben</t>
         </is>
       </c>
     </row>
     <row r="19" ht="22" customHeight="1">
-      <c r="A19" s="8" t="inlineStr">
+      <c r="A19" s="17" t="inlineStr">
         <is>
           <t>Datenbasis</t>
         </is>
       </c>
-      <c r="B19" s="12" t="inlineStr">
+      <c r="B19" s="8" t="inlineStr">
         <is>
           <t>Pilotprogramm CARBOFARM Kft (HU) · 15 Betriebe · 1.500 ha · 3 Jahre historische Daten</t>
-        </is>
-      </c>
-    </row>
-    <row r="20" ht="22" customHeight="1">
-      <c r="A20" s="10" t="inlineStr">
-        <is>
-          <t>Jährl. Ernte</t>
-        </is>
-      </c>
-      <c r="B20" s="14" t="inlineStr">
-        <is>
-          <t>Start nach etabliertem Portfolio und abgeschlossenen Monitoring-Zyklen (je nach Szenario ab 2030)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
fix: wcf = whichever comes first (250 farms OR 100.000 ha)
</commit_message>
<xml_diff>
--- a/GroundUP_BE_Szenarien_2030.xlsx
+++ b/GroundUP_BE_Szenarien_2030.xlsx
@@ -1203,7 +1203,7 @@
       </c>
       <c r="C16" s="8" t="inlineStr">
         <is>
-          <t>Frühjahrsbeprobung 2027 — w.c.f. (1M = 250 Betriebe, worst case figure)</t>
+          <t>Frühjahrsbeprobung 2027 — w.c.f. = whichever comes first (250 Betriebe ODER 100.000 ha — je was zuerst erreicht wird)</t>
         </is>
       </c>
     </row>
@@ -1396,14 +1396,14 @@
     <row r="1" ht="32" customHeight="1">
       <c r="A1" s="12" t="inlineStr">
         <is>
-          <t>Kohorten-Modell — Enrollment-Kaskade 2026–2031 · 50 t netto/Betrieb/2yr-Zyklus (w.c.f.)</t>
+          <t>Kohorten-Modell — Enrollment-Kaskade 2026–2031 · 50 t netto/Betrieb/2yr-Zyklus · w.c.f. = whichever comes first</t>
         </is>
       </c>
     </row>
     <row r="2" ht="22" customHeight="1">
       <c r="A2" s="13" t="inlineStr">
         <is>
-          <t>Enrollment = Baseline + Bodenproben + Laboranalyse + historische Datenaufbereitung je Betrieb  ·  Kohorte zertifiziert nach 2 Jahren Monitoring  ·  1M w.c.f. = 250 Betriebe K1 (Frühjahr 2027)</t>
+          <t>Enrollment = Baseline + Bodenproben + Laboranalyse + historische Datenaufbereitung je Betrieb  ·  Kohorte zertifiziert nach 2 Jahren Monitoring  ·  1M w.c.f. = whichever comes first: 250 Betriebe ODER 100.000 ha (Frühjahr 2027)</t>
         </is>
       </c>
     </row>
@@ -1525,7 +1525,7 @@
       <c r="E6" s="25" t="inlineStr">
         <is>
           <t>125
-Frühjahrsbeprobung 2027 — TREIBER T2 (w.c.f.)</t>
+Frühjahrsbeprobung 2027 — TREIBER T2  (w.c.f.: 250 Betr. od. 100.000 ha)</t>
         </is>
       </c>
       <c r="F6" s="26" t="inlineStr">
@@ -1908,7 +1908,7 @@
       </c>
       <c r="B17" s="35" t="inlineStr">
         <is>
-          <t>2034/2032</t>
+          <t>2032/2034</t>
         </is>
       </c>
       <c r="C17" s="36" t="inlineStr">
@@ -2349,7 +2349,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="69" t="inlineStr">
         <is>
-          <t>500K Regionaler Ausbau  ·  w.c.f. = worst case figure</t>
+          <t>500K Regionaler Ausbau  ·  500K — proportional zur 1M-Basis</t>
         </is>
       </c>
     </row>
@@ -2436,7 +2436,7 @@
       </c>
       <c r="F7" s="74" t="inlineStr">
         <is>
-          <t>Frühjahrsbeprobung 2027 — TREIBER T2 (w.c.f.)</t>
+          <t>Frühjahrsbeprobung 2027 — TREIBER T2  (w.c.f.: 250 Betr. od. 100.000 ha)</t>
         </is>
       </c>
     </row>
@@ -2745,7 +2745,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="80" t="inlineStr">
         <is>
-          <t>1M AT-Exklusivität  ·  w.c.f. = worst case figure</t>
+          <t>1M AT-Exklusivität  ·  w.c.f. = whichever comes first (250 Betr. / 100.000 ha)</t>
         </is>
       </c>
     </row>

</xml_diff>